<commit_message>
Agrega banner de auspiciadores en la portada
- Nueva pestaña Auspiciadores en datos.xlsx (orden, nombre, imagen,
  url opcional) y su función getAuspiciadores() en lib/datos.ts
- Nuevo componente AuspiciadoresBanner: fila de logos bajo el
  carrusel de la portada, sin recortar (object-contain), cada uno
  clicable a su sitio si tiene url; no muestra nada si no hay
  auspiciadores cargados
- Nueva carpeta public/auspiciadores/ para los logos
- Suma la carpeta a la sincronización automática (sincronizar.gs +
  AUTOMATIZACION.md) y documenta la pestaña/carpeta en el README
</commit_message>
<xml_diff>
--- a/data/datos.xlsx
+++ b/data/datos.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Calendario" sheetId="8" r:id="rId8"/>
     <sheet name="Novedades" sheetId="9" r:id="rId9"/>
     <sheet name="Galeria" sheetId="10" r:id="rId10"/>
+    <sheet name="Auspiciadores" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -709,6 +710,31 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>orden</v>
+      </c>
+      <c r="B1" t="str">
+        <v>nombre</v>
+      </c>
+      <c r="C1" t="str">
+        <v>imagen</v>
+      </c>
+      <c r="D1" t="str">
+        <v>url</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C6"/>

</xml_diff>